<commit_message>
Ajout player + animation idle + animation walk+ mouvement gauche droite
</commit_message>
<xml_diff>
--- a/TP02_Taches.xlsx
+++ b/TP02_Taches.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Administrateur.UTILISA-UKLTCCH\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\__Projet_Jeux_videos\projet_platformer_tp2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2A77FB-55A2-4A25-8D18-B0BBBDDB1AF6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC10310B-6839-418B-97E2-695E88CF09AA}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tâches" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tâches!$A$1:$E$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="105">
   <si>
     <t>Catégorie</t>
   </si>
@@ -334,13 +334,22 @@
   </si>
   <si>
     <t>Vérifier durée 1-2 min, équilibrage, qu’on peut finir le niveau.</t>
+  </si>
+  <si>
+    <t>Eddy</t>
+  </si>
+  <si>
+    <t>Antoine</t>
+  </si>
+  <si>
+    <t>Fait</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -365,8 +374,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -439,6 +460,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -480,7 +507,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -520,6 +547,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -786,16 +822,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="23.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
-    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.90625" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.88671875" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -812,7 +848,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -825,9 +861,11 @@
       <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E2" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -840,9 +878,11 @@
       <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E3" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -855,9 +895,11 @@
       <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E4" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -870,9 +912,11 @@
       <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E5" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
@@ -885,9 +929,11 @@
       <c r="D6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E6" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>15</v>
       </c>
@@ -900,9 +946,11 @@
       <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E7" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
@@ -915,9 +963,11 @@
       <c r="D8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
@@ -930,9 +980,9 @@
       <c r="D9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E9" s="14"/>
+    </row>
+    <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>21</v>
       </c>
@@ -945,9 +995,9 @@
       <c r="D10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E10" s="14"/>
+    </row>
+    <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
@@ -960,9 +1010,9 @@
       <c r="D11" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E11" s="14"/>
+    </row>
+    <row r="12" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
@@ -975,9 +1025,9 @@
       <c r="D12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E12" s="14"/>
+    </row>
+    <row r="13" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>28</v>
       </c>
@@ -990,9 +1040,9 @@
       <c r="D13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E13" s="14"/>
+    </row>
+    <row r="14" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>28</v>
       </c>
@@ -1005,9 +1055,9 @@
       <c r="D14" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E14" s="14"/>
+    </row>
+    <row r="15" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>35</v>
       </c>
@@ -1020,9 +1070,9 @@
       <c r="D15" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E15" s="14"/>
+    </row>
+    <row r="16" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>35</v>
       </c>
@@ -1035,9 +1085,9 @@
       <c r="D16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>35</v>
       </c>
@@ -1050,9 +1100,9 @@
       <c r="D17" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E17" s="14"/>
+    </row>
+    <row r="18" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>35</v>
       </c>
@@ -1065,9 +1115,9 @@
       <c r="D18" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E18" s="14"/>
+    </row>
+    <row r="19" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>35</v>
       </c>
@@ -1080,9 +1130,9 @@
       <c r="D19" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E19" s="14"/>
+    </row>
+    <row r="20" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>35</v>
       </c>
@@ -1095,9 +1145,9 @@
       <c r="D20" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>35</v>
       </c>
@@ -1110,9 +1160,9 @@
       <c r="D21" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E21" s="14"/>
+    </row>
+    <row r="22" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>50</v>
       </c>
@@ -1123,9 +1173,11 @@
       <c r="D22" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E22" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>50</v>
       </c>
@@ -1138,9 +1190,11 @@
       <c r="D23" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E23" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>50</v>
       </c>
@@ -1153,9 +1207,11 @@
       <c r="D24" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E24" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>50</v>
       </c>
@@ -1165,12 +1221,14 @@
       <c r="C25" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D25" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>50</v>
       </c>
@@ -1178,12 +1236,14 @@
         <v>58</v>
       </c>
       <c r="C26" s="2"/>
-      <c r="D26" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D26" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>50</v>
       </c>
@@ -1194,9 +1254,11 @@
       <c r="D27" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E27" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>50</v>
       </c>
@@ -1209,9 +1271,11 @@
       <c r="D28" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E28" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>50</v>
       </c>
@@ -1222,9 +1286,11 @@
       <c r="D29" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E29" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>50</v>
       </c>
@@ -1232,12 +1298,14 @@
         <v>63</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="D30" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D30" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>50</v>
       </c>
@@ -1248,9 +1316,11 @@
       <c r="D31" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E31" s="2"/>
-    </row>
-    <row r="32" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E31" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>50</v>
       </c>
@@ -1261,9 +1331,11 @@
       <c r="D32" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E32" s="2"/>
-    </row>
-    <row r="33" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E32" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>50</v>
       </c>
@@ -1274,9 +1346,11 @@
       <c r="D33" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E33" s="2"/>
-    </row>
-    <row r="34" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E33" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>50</v>
       </c>
@@ -1287,9 +1361,11 @@
       <c r="D34" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E34" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>68</v>
       </c>
@@ -1302,9 +1378,9 @@
       <c r="D35" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E35" s="2"/>
-    </row>
-    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E35" s="14"/>
+    </row>
+    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>68</v>
       </c>
@@ -1317,9 +1393,9 @@
       <c r="D36" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E36" s="2"/>
-    </row>
-    <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E36" s="14"/>
+    </row>
+    <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="13" t="s">
         <v>73</v>
       </c>
@@ -1332,9 +1408,9 @@
       <c r="D37" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E37" s="2"/>
-    </row>
-    <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E37" s="14"/>
+    </row>
+    <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>73</v>
       </c>
@@ -1347,9 +1423,9 @@
       <c r="D38" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E38" s="2"/>
-    </row>
-    <row r="39" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E38" s="14"/>
+    </row>
+    <row r="39" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
         <v>73</v>
       </c>
@@ -1362,9 +1438,9 @@
       <c r="D39" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E39" s="2"/>
-    </row>
-    <row r="40" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E39" s="14"/>
+    </row>
+    <row r="40" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>73</v>
       </c>
@@ -1377,9 +1453,9 @@
       <c r="D40" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E40" s="2"/>
-    </row>
-    <row r="41" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E40" s="14"/>
+    </row>
+    <row r="41" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>73</v>
       </c>
@@ -1392,9 +1468,9 @@
       <c r="D41" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="2"/>
-    </row>
-    <row r="42" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E41" s="14"/>
+    </row>
+    <row r="42" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>73</v>
       </c>
@@ -1407,9 +1483,9 @@
       <c r="D42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E42" s="2"/>
-    </row>
-    <row r="43" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E42" s="14"/>
+    </row>
+    <row r="43" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
         <v>73</v>
       </c>
@@ -1422,9 +1498,9 @@
       <c r="D43" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E43" s="2"/>
-    </row>
-    <row r="44" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E43" s="14"/>
+    </row>
+    <row r="44" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>88</v>
       </c>
@@ -1437,9 +1513,9 @@
       <c r="D44" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E44" s="2"/>
-    </row>
-    <row r="45" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E44" s="14"/>
+    </row>
+    <row r="45" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>88</v>
       </c>
@@ -1452,9 +1528,9 @@
       <c r="D45" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E45" s="14"/>
+    </row>
+    <row r="46" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>92</v>
       </c>
@@ -1467,9 +1543,9 @@
       <c r="D46" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E46" s="2"/>
-    </row>
-    <row r="47" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E46" s="14"/>
+    </row>
+    <row r="47" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>92</v>
       </c>
@@ -1480,9 +1556,9 @@
       <c r="D47" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E47" s="2"/>
-    </row>
-    <row r="48" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E47" s="14"/>
+    </row>
+    <row r="48" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>92</v>
       </c>
@@ -1493,9 +1569,9 @@
       <c r="D48" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E48" s="14"/>
+    </row>
+    <row r="49" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
         <v>97</v>
       </c>
@@ -1508,9 +1584,9 @@
       <c r="D49" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E49" s="14"/>
+    </row>
+    <row r="50" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
         <v>97</v>
       </c>
@@ -1523,7 +1599,7 @@
       <c r="D50" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E50" s="2"/>
+      <c r="E50" s="14"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{26CE1A3D-2936-48E9-B7C5-23539BB9D800}"/>

</xml_diff>

<commit_message>
Ajout player Dash+ animation + fix  flip sprite au départ
</commit_message>
<xml_diff>
--- a/TP02_Taches.xlsx
+++ b/TP02_Taches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\__Projet_Jeux_videos\projet_platformer_tp2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CE0844-0E06-42A0-94EE-36717777EDDE}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D7505-12F2-40A6-B608-ABCF59EAEFCC}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="105">
   <si>
     <t>Catégorie</t>
   </si>
@@ -294,9 +294,6 @@
     <t>Saute sur place. Tire un projectile de temps en temps. 5 PV. Animations sur place + saut.</t>
   </si>
   <si>
-    <t>Interface</t>
-  </si>
-  <si>
     <t>Barre de vie rouge</t>
   </si>
   <si>
@@ -343,6 +340,9 @@
   </si>
   <si>
     <t>Fait</t>
+  </si>
+  <si>
+    <t>Charlotte</t>
   </si>
 </sst>
 </file>
@@ -862,7 +862,7 @@
         <v>5</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -879,7 +879,7 @@
         <v>5</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -896,7 +896,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -913,7 +913,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -930,7 +930,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -947,7 +947,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -964,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1170,11 +1170,11 @@
         <v>51</v>
       </c>
       <c r="C22" s="2"/>
-      <c r="D22" s="3" t="s">
-        <v>5</v>
+      <c r="D22" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1182,16 +1182,16 @@
         <v>50</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>5</v>
+        <v>57</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1199,16 +1199,14 @@
         <v>50</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>5</v>
+        <v>58</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1216,16 +1214,16 @@
         <v>50</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>5</v>
+        <v>103</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1233,14 +1231,14 @@
         <v>50</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1248,14 +1246,14 @@
         <v>50</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C27" s="2"/>
-      <c r="D27" s="3" t="s">
-        <v>5</v>
+      <c r="D27" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1263,16 +1261,14 @@
         <v>50</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>61</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="C28" s="2"/>
       <c r="D28" s="16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1280,14 +1276,14 @@
         <v>50</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C29" s="2"/>
-      <c r="D29" s="3" t="s">
-        <v>5</v>
+      <c r="D29" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1295,14 +1291,14 @@
         <v>50</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="D30" s="16" t="s">
-        <v>104</v>
+      <c r="D30" s="3" t="s">
+        <v>5</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1310,14 +1306,16 @@
         <v>50</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="16" t="s">
-        <v>104</v>
+        <v>52</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>5</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1325,14 +1323,16 @@
         <v>50</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="D32" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1347,7 +1347,7 @@
         <v>5</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1362,41 +1362,41 @@
         <v>5</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="C36" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1413,7 +1413,7 @@
         <v>5</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1430,7 +1430,7 @@
         <v>5</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1446,7 +1446,9 @@
       <c r="D39" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E39" s="14"/>
+      <c r="E39" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="40" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
@@ -1461,7 +1463,9 @@
       <c r="D40" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E40" s="14"/>
+      <c r="E40" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="41" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
@@ -1476,7 +1480,9 @@
       <c r="D41" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="14"/>
+      <c r="E41" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="42" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
@@ -1491,7 +1497,9 @@
       <c r="D42" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E42" s="14"/>
+      <c r="E42" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="43" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="13" t="s">
@@ -1506,7 +1514,9 @@
       <c r="D43" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E43" s="14"/>
+      <c r="E43" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="44" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
@@ -1521,7 +1531,9 @@
       <c r="D44" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E44" s="14"/>
+      <c r="E44" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="45" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="13" t="s">
@@ -1536,17 +1548,19 @@
       <c r="D45" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E45" s="14"/>
+      <c r="E45" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="46" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>5</v>
@@ -1555,10 +1569,10 @@
     </row>
     <row r="47" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="3" t="s">
@@ -1568,10 +1582,10 @@
     </row>
     <row r="48" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="3" t="s">
@@ -1581,13 +1595,13 @@
     </row>
     <row r="49" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>5</v>
@@ -1596,13 +1610,13 @@
     </row>
     <row r="50" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Ajout joueur : clique souris+ animation tir
</commit_message>
<xml_diff>
--- a/TP02_Taches.xlsx
+++ b/TP02_Taches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\__Projet_Jeux_videos\projet_platformer_tp2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D7505-12F2-40A6-B608-ABCF59EAEFCC}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9426C6-17CD-4118-9A94-2DA21D002EA6}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="106">
   <si>
     <t>Catégorie</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>Charlotte</t>
+  </si>
+  <si>
+    <t>En cours</t>
   </si>
 </sst>
 </file>
@@ -387,7 +390,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -466,6 +469,12 @@
         <bgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -507,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -555,6 +564,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1287,29 +1299,31 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="6" t="s">
-        <v>50</v>
+      <c r="A30" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="3" t="s">
-        <v>5</v>
+        <v>69</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>105</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="6" t="s">
-        <v>50</v>
+      <c r="A31" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>5</v>
@@ -1323,11 +1337,9 @@
         <v>50</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>55</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="C32" s="2"/>
       <c r="D32" s="3" t="s">
         <v>5</v>
       </c>
@@ -1340,7 +1352,7 @@
         <v>50</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="3" t="s">
@@ -1355,9 +1367,11 @@
         <v>50</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D34" s="3" t="s">
         <v>5</v>
       </c>
@@ -1370,10 +1384,10 @@
         <v>50</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>5</v>
@@ -1387,11 +1401,9 @@
         <v>50</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>89</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="C36" s="2"/>
       <c r="D36" s="3" t="s">
         <v>5</v>
       </c>
@@ -1400,14 +1412,14 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
-        <v>68</v>
+      <c r="A37" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>5</v>
@@ -1417,14 +1429,14 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="9" t="s">
-        <v>68</v>
+      <c r="A38" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Avancement dans la construction du niveau un.
</commit_message>
<xml_diff>
--- a/TP02_Taches.xlsx
+++ b/TP02_Taches.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\__Projet_Jeux_videos\projet_platformer_tp2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\projet_platformer_tp2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9426C6-17CD-4118-9A94-2DA21D002EA6}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E2CC88-2981-403C-86E1-B7FD9283B594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tâches" sheetId="1" r:id="rId1"/>
@@ -834,16 +834,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="23.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="23.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.88671875" style="15" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.85546875" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -860,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -877,7 +877,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -894,7 +894,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -911,7 +911,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -928,7 +928,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
@@ -945,7 +945,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>15</v>
       </c>
@@ -962,7 +962,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
@@ -979,7 +979,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
@@ -994,7 +994,7 @@
       </c>
       <c r="E9" s="14"/>
     </row>
-    <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>21</v>
       </c>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="E10" s="14"/>
     </row>
-    <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>21</v>
       </c>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="E11" s="14"/>
     </row>
-    <row r="12" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E12" s="14"/>
     </row>
-    <row r="13" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>28</v>
       </c>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="E13" s="14"/>
     </row>
-    <row r="14" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>28</v>
       </c>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="E14" s="14"/>
     </row>
-    <row r="15" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>35</v>
       </c>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="E15" s="14"/>
     </row>
-    <row r="16" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>35</v>
       </c>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E16" s="14"/>
     </row>
-    <row r="17" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>35</v>
       </c>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E17" s="14"/>
     </row>
-    <row r="18" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>35</v>
       </c>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="E18" s="14"/>
     </row>
-    <row r="19" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>35</v>
       </c>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E19" s="14"/>
     </row>
-    <row r="20" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>35</v>
       </c>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E20" s="14"/>
     </row>
-    <row r="21" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>35</v>
       </c>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="E21" s="14"/>
     </row>
-    <row r="22" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>50</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>50</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>50</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>50</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>50</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>50</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>50</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>50</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>68</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>68</v>
       </c>
@@ -1332,7 +1332,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>50</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>50</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>50</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>50</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>50</v>
       </c>
@@ -1411,7 +1411,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>50</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>50</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>73</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>73</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
         <v>73</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
         <v>73</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>73</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>73</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>73</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>91</v>
       </c>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E46" s="14"/>
     </row>
-    <row r="47" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>91</v>
       </c>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E47" s="14"/>
     </row>
-    <row r="48" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>91</v>
       </c>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="E48" s="14"/>
     </row>
-    <row r="49" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>96</v>
       </c>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="E49" s="14"/>
     </row>
-    <row r="50" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
         <v>96</v>
       </c>

</xml_diff>